<commit_message>
feat: populate gender, birth_date, and address fields on free user accounts
</commit_message>
<xml_diff>
--- a/danh_sach_tai_khoan.xlsx
+++ b/danh_sach_tai_khoan.xlsx
@@ -458,7 +458,7 @@
         <v>free</v>
       </c>
       <c r="H2" t="str">
-        <v>19:44:22 23/5/2026</v>
+        <v>04:56:21 24/5/2026</v>
       </c>
     </row>
     <row r="3">
@@ -484,7 +484,7 @@
         <v>free</v>
       </c>
       <c r="H3" t="str">
-        <v>01:49:25 3/6/2026</v>
+        <v>19:10:37 2/6/2026</v>
       </c>
     </row>
     <row r="4">
@@ -510,7 +510,7 @@
         <v>free</v>
       </c>
       <c r="H4" t="str">
-        <v>04:36:59 13/6/2026</v>
+        <v>18:25:44 12/6/2026</v>
       </c>
     </row>
     <row r="5">
@@ -536,7 +536,7 @@
         <v>free</v>
       </c>
       <c r="H5" t="str">
-        <v>20:36:36 17/6/2026</v>
+        <v>23:32:32 17/6/2026</v>
       </c>
     </row>
     <row r="6">
@@ -562,7 +562,7 @@
         <v>free</v>
       </c>
       <c r="H6" t="str">
-        <v>02:48:19 24/5/2026</v>
+        <v>23:22:14 23/5/2026</v>
       </c>
     </row>
     <row r="7">
@@ -588,7 +588,7 @@
         <v>free</v>
       </c>
       <c r="H7" t="str">
-        <v>01:24:10 3/6/2026</v>
+        <v>02:07:00 3/6/2026</v>
       </c>
     </row>
     <row r="8">
@@ -614,7 +614,7 @@
         <v>free</v>
       </c>
       <c r="H8" t="str">
-        <v>00:51:13 13/6/2026</v>
+        <v>20:03:35 12/6/2026</v>
       </c>
     </row>
     <row r="9">
@@ -640,7 +640,7 @@
         <v>free</v>
       </c>
       <c r="H9" t="str">
-        <v>00:26:06 18/6/2026</v>
+        <v>21:31:42 17/6/2026</v>
       </c>
     </row>
     <row r="10">
@@ -666,7 +666,7 @@
         <v>free</v>
       </c>
       <c r="H10" t="str">
-        <v>05:00:24 24/5/2026</v>
+        <v>19:12:30 23/5/2026</v>
       </c>
     </row>
     <row r="11">
@@ -692,7 +692,7 @@
         <v>free</v>
       </c>
       <c r="H11" t="str">
-        <v>23:26:36 2/6/2026</v>
+        <v>22:28:52 2/6/2026</v>
       </c>
     </row>
     <row r="12">
@@ -718,7 +718,7 @@
         <v>free</v>
       </c>
       <c r="H12" t="str">
-        <v>22:21:44 12/6/2026</v>
+        <v>04:32:53 13/6/2026</v>
       </c>
     </row>
     <row r="13">
@@ -744,7 +744,7 @@
         <v>free</v>
       </c>
       <c r="H13" t="str">
-        <v>22:31:56 17/6/2026</v>
+        <v>23:28:23 17/6/2026</v>
       </c>
     </row>
     <row r="14">
@@ -770,7 +770,7 @@
         <v>free</v>
       </c>
       <c r="H14" t="str">
-        <v>21:29:34 23/5/2026</v>
+        <v>17:38:56 23/5/2026</v>
       </c>
     </row>
     <row r="15">
@@ -796,7 +796,7 @@
         <v>free</v>
       </c>
       <c r="H15" t="str">
-        <v>00:02:17 3/6/2026</v>
+        <v>22:00:38 2/6/2026</v>
       </c>
     </row>
     <row r="16">
@@ -822,7 +822,7 @@
         <v>free</v>
       </c>
       <c r="H16" t="str">
-        <v>23:14:50 12/6/2026</v>
+        <v>18:06:40 12/6/2026</v>
       </c>
     </row>
     <row r="17">
@@ -848,7 +848,7 @@
         <v>free</v>
       </c>
       <c r="H17" t="str">
-        <v>20:23:19 17/6/2026</v>
+        <v>01:52:39 18/6/2026</v>
       </c>
     </row>
     <row r="18">
@@ -874,7 +874,7 @@
         <v>free</v>
       </c>
       <c r="H18" t="str">
-        <v>22:33:00 23/5/2026</v>
+        <v>21:11:29 23/5/2026</v>
       </c>
     </row>
     <row r="19">
@@ -900,7 +900,7 @@
         <v>free</v>
       </c>
       <c r="H19" t="str">
-        <v>04:27:27 3/6/2026</v>
+        <v>22:21:14 2/6/2026</v>
       </c>
     </row>
     <row r="20">
@@ -926,7 +926,7 @@
         <v>free</v>
       </c>
       <c r="H20" t="str">
-        <v>23:28:46 12/6/2026</v>
+        <v>02:33:56 13/6/2026</v>
       </c>
     </row>
     <row r="21">
@@ -952,7 +952,7 @@
         <v>free</v>
       </c>
       <c r="H21" t="str">
-        <v>01:33:46 18/6/2026</v>
+        <v>02:23:10 18/6/2026</v>
       </c>
     </row>
     <row r="22">
@@ -978,7 +978,7 @@
         <v>free</v>
       </c>
       <c r="H22" t="str">
-        <v>19:26:00 23/5/2026</v>
+        <v>03:05:10 24/5/2026</v>
       </c>
     </row>
     <row r="23">
@@ -1004,7 +1004,7 @@
         <v>free</v>
       </c>
       <c r="H23" t="str">
-        <v>18:57:58 2/6/2026</v>
+        <v>01:39:42 3/6/2026</v>
       </c>
     </row>
     <row r="24">
@@ -1030,7 +1030,7 @@
         <v>free</v>
       </c>
       <c r="H24" t="str">
-        <v>19:27:34 12/6/2026</v>
+        <v>01:43:55 13/6/2026</v>
       </c>
     </row>
     <row r="25">
@@ -1056,7 +1056,7 @@
         <v>free</v>
       </c>
       <c r="H25" t="str">
-        <v>04:42:28 18/6/2026</v>
+        <v>05:04:25 18/6/2026</v>
       </c>
     </row>
     <row r="26">
@@ -1082,7 +1082,7 @@
         <v>free</v>
       </c>
       <c r="H26" t="str">
-        <v>00:23:49 24/5/2026</v>
+        <v>19:58:39 23/5/2026</v>
       </c>
     </row>
     <row r="27">
@@ -1108,7 +1108,7 @@
         <v>free</v>
       </c>
       <c r="H27" t="str">
-        <v>21:43:38 2/6/2026</v>
+        <v>04:35:32 3/6/2026</v>
       </c>
     </row>
     <row r="28">
@@ -1134,7 +1134,7 @@
         <v>free</v>
       </c>
       <c r="H28" t="str">
-        <v>22:47:58 12/6/2026</v>
+        <v>03:05:31 13/6/2026</v>
       </c>
     </row>
     <row r="29">
@@ -1160,7 +1160,7 @@
         <v>free</v>
       </c>
       <c r="H29" t="str">
-        <v>19:36:21 17/6/2026</v>
+        <v>02:26:16 18/6/2026</v>
       </c>
     </row>
     <row r="30">
@@ -1186,7 +1186,7 @@
         <v>free</v>
       </c>
       <c r="H30" t="str">
-        <v>01:08:18 24/5/2026</v>
+        <v>23:43:21 23/5/2026</v>
       </c>
     </row>
     <row r="31">
@@ -1212,7 +1212,7 @@
         <v>free</v>
       </c>
       <c r="H31" t="str">
-        <v>23:18:51 2/6/2026</v>
+        <v>18:44:48 2/6/2026</v>
       </c>
     </row>
     <row r="32">
@@ -1238,7 +1238,7 @@
         <v>free</v>
       </c>
       <c r="H32" t="str">
-        <v>20:44:49 12/6/2026</v>
+        <v>04:24:19 13/6/2026</v>
       </c>
     </row>
     <row r="33">
@@ -1264,7 +1264,7 @@
         <v>free</v>
       </c>
       <c r="H33" t="str">
-        <v>23:11:14 17/6/2026</v>
+        <v>00:43:08 18/6/2026</v>
       </c>
     </row>
     <row r="34">
@@ -1290,7 +1290,7 @@
         <v>free</v>
       </c>
       <c r="H34" t="str">
-        <v>23:34:11 23/5/2026</v>
+        <v>22:34:44 23/5/2026</v>
       </c>
     </row>
     <row r="35">
@@ -1316,7 +1316,7 @@
         <v>free</v>
       </c>
       <c r="H35" t="str">
-        <v>18:58:34 2/6/2026</v>
+        <v>01:07:43 3/6/2026</v>
       </c>
     </row>
     <row r="36">
@@ -1342,7 +1342,7 @@
         <v>free</v>
       </c>
       <c r="H36" t="str">
-        <v>19:32:30 12/6/2026</v>
+        <v>01:34:11 13/6/2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add address, gender, and birth date to free user excel report
</commit_message>
<xml_diff>
--- a/danh_sach_tai_khoan.xlsx
+++ b/danh_sach_tai_khoan.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:K36"/>
   <cols>
     <col min="1" max="1"/>
     <col min="2" max="2"/>
@@ -407,6 +407,9 @@
     <col min="6" max="6"/>
     <col min="7" max="7"/>
     <col min="8" max="8"/>
+    <col min="9" max="9"/>
+    <col min="10" max="10"/>
+    <col min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,18 +423,27 @@
         <v>Tuổi Bé</v>
       </c>
       <c r="D1" t="str">
+        <v>Giới tính</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Ngày sinh</v>
+      </c>
+      <c r="F1" t="str">
         <v>Họ và Tên Bố Mẹ</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Tuổi Bố Mẹ</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
+        <v>Địa chỉ</v>
+      </c>
+      <c r="I1" t="str">
         <v>Email</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>Loại tài khoản</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>Ngày tạo nick</v>
       </c>
     </row>
@@ -446,19 +458,28 @@
         <v>5</v>
       </c>
       <c r="D2" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2021-07-26</v>
+      </c>
+      <c r="F2" t="str">
         <v>Nguyễn Văn Hùng</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>35</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
+        <v>Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I2" t="str">
         <v>hung.nguyenvan.1991@gmail.com</v>
       </c>
-      <c r="G2" t="str">
-        <v>free</v>
-      </c>
-      <c r="H2" t="str">
-        <v>04:56:21 24/5/2026</v>
+      <c r="J2" t="str">
+        <v>free</v>
+      </c>
+      <c r="K2" t="str">
+        <v>23:13:55 23/5/2026</v>
       </c>
     </row>
     <row r="3">
@@ -472,19 +493,28 @@
         <v>6</v>
       </c>
       <c r="D3" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2020-08-28</v>
+      </c>
+      <c r="F3" t="str">
         <v>Trần Quốc Anh</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>36</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
+        <v>Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I3" t="str">
         <v>anh.tranquoc.1990@yahoo.com</v>
       </c>
-      <c r="G3" t="str">
-        <v>free</v>
-      </c>
-      <c r="H3" t="str">
-        <v>19:10:37 2/6/2026</v>
+      <c r="J3" t="str">
+        <v>free</v>
+      </c>
+      <c r="K3" t="str">
+        <v>03:10:26 3/6/2026</v>
       </c>
     </row>
     <row r="4">
@@ -498,19 +528,28 @@
         <v>7</v>
       </c>
       <c r="D4" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2019-05-12</v>
+      </c>
+      <c r="F4" t="str">
         <v>Lê Văn Hải</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>37</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
+        <v>TX. Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I4" t="str">
         <v>hai.levan.1989@outlook.com</v>
       </c>
-      <c r="G4" t="str">
-        <v>free</v>
-      </c>
-      <c r="H4" t="str">
-        <v>18:25:44 12/6/2026</v>
+      <c r="J4" t="str">
+        <v>free</v>
+      </c>
+      <c r="K4" t="str">
+        <v>03:36:00 13/6/2026</v>
       </c>
     </row>
     <row r="5">
@@ -524,19 +563,28 @@
         <v>8</v>
       </c>
       <c r="D5" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2018-03-16</v>
+      </c>
+      <c r="F5" t="str">
         <v>Phạm Thanh Sơn</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>38</v>
       </c>
-      <c r="F5" t="str">
+      <c r="H5" t="str">
+        <v>H. Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I5" t="str">
         <v>son.phamthanh.1988@hotmail.com</v>
       </c>
-      <c r="G5" t="str">
-        <v>free</v>
-      </c>
-      <c r="H5" t="str">
-        <v>23:32:32 17/6/2026</v>
+      <c r="J5" t="str">
+        <v>free</v>
+      </c>
+      <c r="K5" t="str">
+        <v>20:36:03 17/6/2026</v>
       </c>
     </row>
     <row r="6">
@@ -550,19 +598,28 @@
         <v>9</v>
       </c>
       <c r="D6" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2017-04-19</v>
+      </c>
+      <c r="F6" t="str">
         <v>Hoàng Minh Đức</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>39</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
+        <v>Phường Ngô Quyền, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I6" t="str">
         <v>duc.hoangminh.1987@fpt.edu.vn</v>
       </c>
-      <c r="G6" t="str">
-        <v>free</v>
-      </c>
-      <c r="H6" t="str">
-        <v>23:22:14 23/5/2026</v>
+      <c r="J6" t="str">
+        <v>free</v>
+      </c>
+      <c r="K6" t="str">
+        <v>18:38:40 23/5/2026</v>
       </c>
     </row>
     <row r="7">
@@ -576,19 +633,28 @@
         <v>10</v>
       </c>
       <c r="D7" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2016-07-03</v>
+      </c>
+      <c r="F7" t="str">
         <v>Huỳnh Anh Tuấn</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>40</v>
       </c>
-      <c r="F7" t="str">
+      <c r="H7" t="str">
+        <v>Xã Bình Yên, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I7" t="str">
         <v>tuan.huynhanh.1986@gmail.com</v>
       </c>
-      <c r="G7" t="str">
-        <v>free</v>
-      </c>
-      <c r="H7" t="str">
-        <v>02:07:00 3/6/2026</v>
+      <c r="J7" t="str">
+        <v>free</v>
+      </c>
+      <c r="K7" t="str">
+        <v>00:48:06 3/6/2026</v>
       </c>
     </row>
     <row r="8">
@@ -602,19 +668,28 @@
         <v>11</v>
       </c>
       <c r="D8" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2015-03-28</v>
+      </c>
+      <c r="F8" t="str">
         <v>Phan Văn Hoàng</v>
       </c>
-      <c r="E8">
+      <c r="G8">
         <v>35</v>
       </c>
-      <c r="F8" t="str">
+      <c r="H8" t="str">
+        <v>Phường Quang Trung, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I8" t="str">
         <v>hoang.phanvan.1991@yahoo.com</v>
       </c>
-      <c r="G8" t="str">
-        <v>free</v>
-      </c>
-      <c r="H8" t="str">
-        <v>20:03:35 12/6/2026</v>
+      <c r="J8" t="str">
+        <v>free</v>
+      </c>
+      <c r="K8" t="str">
+        <v>22:33:55 12/6/2026</v>
       </c>
     </row>
     <row r="9">
@@ -628,19 +703,28 @@
         <v>12</v>
       </c>
       <c r="D9" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2014-09-15</v>
+      </c>
+      <c r="F9" t="str">
         <v>Vũ Minh Tiến</v>
       </c>
-      <c r="E9">
+      <c r="G9">
         <v>36</v>
       </c>
-      <c r="F9" t="str">
+      <c r="H9" t="str">
+        <v>Xã Liên Quan, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I9" t="str">
         <v>tien.vuminh.1990@outlook.com</v>
       </c>
-      <c r="G9" t="str">
-        <v>free</v>
-      </c>
-      <c r="H9" t="str">
-        <v>21:31:42 17/6/2026</v>
+      <c r="J9" t="str">
+        <v>free</v>
+      </c>
+      <c r="K9" t="str">
+        <v>20:56:47 17/6/2026</v>
       </c>
     </row>
     <row r="10">
@@ -654,19 +738,28 @@
         <v>5</v>
       </c>
       <c r="D10" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2021-09-25</v>
+      </c>
+      <c r="F10" t="str">
         <v>Võ Văn Nam</v>
       </c>
-      <c r="E10">
+      <c r="G10">
         <v>37</v>
       </c>
-      <c r="F10" t="str">
+      <c r="H10" t="str">
+        <v>Phường Lê Lợi, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I10" t="str">
         <v>nam.vovan.1989@hotmail.com</v>
       </c>
-      <c r="G10" t="str">
-        <v>free</v>
-      </c>
-      <c r="H10" t="str">
-        <v>19:12:30 23/5/2026</v>
+      <c r="J10" t="str">
+        <v>free</v>
+      </c>
+      <c r="K10" t="str">
+        <v>03:14:50 24/5/2026</v>
       </c>
     </row>
     <row r="11">
@@ -680,19 +773,28 @@
         <v>6</v>
       </c>
       <c r="D11" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2020-04-10</v>
+      </c>
+      <c r="F11" t="str">
         <v>Đặng Quốc Khánh</v>
       </c>
-      <c r="E11">
+      <c r="G11">
         <v>38</v>
       </c>
-      <c r="F11" t="str">
+      <c r="H11" t="str">
+        <v>Xã Kim Quan, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I11" t="str">
         <v>khanh.dangquoc.1988@fpt.edu.vn</v>
       </c>
-      <c r="G11" t="str">
-        <v>free</v>
-      </c>
-      <c r="H11" t="str">
-        <v>22:28:52 2/6/2026</v>
+      <c r="J11" t="str">
+        <v>free</v>
+      </c>
+      <c r="K11" t="str">
+        <v>21:33:35 2/6/2026</v>
       </c>
     </row>
     <row r="12">
@@ -706,19 +808,28 @@
         <v>7</v>
       </c>
       <c r="D12" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2019-09-21</v>
+      </c>
+      <c r="F12" t="str">
         <v>Bùi Hồng Sơn</v>
       </c>
-      <c r="E12">
+      <c r="G12">
         <v>39</v>
       </c>
-      <c r="F12" t="str">
+      <c r="H12" t="str">
+        <v>Phường Sơn Lộc, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I12" t="str">
         <v>son.buihong.1987@gmail.com</v>
       </c>
-      <c r="G12" t="str">
-        <v>free</v>
-      </c>
-      <c r="H12" t="str">
-        <v>04:32:53 13/6/2026</v>
+      <c r="J12" t="str">
+        <v>free</v>
+      </c>
+      <c r="K12" t="str">
+        <v>01:41:24 13/6/2026</v>
       </c>
     </row>
     <row r="13">
@@ -732,19 +843,28 @@
         <v>8</v>
       </c>
       <c r="D13" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2018-08-27</v>
+      </c>
+      <c r="F13" t="str">
         <v>Đỗ Minh Quân</v>
       </c>
-      <c r="E13">
+      <c r="G13">
         <v>40</v>
       </c>
-      <c r="F13" t="str">
+      <c r="H13" t="str">
+        <v>Xã Phùng Xá, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I13" t="str">
         <v>quan.dominh.1986@yahoo.com</v>
       </c>
-      <c r="G13" t="str">
-        <v>free</v>
-      </c>
-      <c r="H13" t="str">
-        <v>23:28:23 17/6/2026</v>
+      <c r="J13" t="str">
+        <v>free</v>
+      </c>
+      <c r="K13" t="str">
+        <v>20:49:32 17/6/2026</v>
       </c>
     </row>
     <row r="14">
@@ -758,19 +878,28 @@
         <v>9</v>
       </c>
       <c r="D14" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2017-04-05</v>
+      </c>
+      <c r="F14" t="str">
         <v>Ngô Văn Hùng</v>
       </c>
-      <c r="E14">
+      <c r="G14">
         <v>35</v>
       </c>
-      <c r="F14" t="str">
+      <c r="H14" t="str">
+        <v>Phường Trung Hưng, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I14" t="str">
         <v>hung.ngovan.1991@outlook.com</v>
       </c>
-      <c r="G14" t="str">
-        <v>free</v>
-      </c>
-      <c r="H14" t="str">
-        <v>17:38:56 23/5/2026</v>
+      <c r="J14" t="str">
+        <v>free</v>
+      </c>
+      <c r="K14" t="str">
+        <v>18:56:08 23/5/2026</v>
       </c>
     </row>
     <row r="15">
@@ -784,19 +913,28 @@
         <v>10</v>
       </c>
       <c r="D15" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2016-06-10</v>
+      </c>
+      <c r="F15" t="str">
         <v>Dương Minh Hoàng</v>
       </c>
-      <c r="E15">
+      <c r="G15">
         <v>36</v>
       </c>
-      <c r="F15" t="str">
+      <c r="H15" t="str">
+        <v>Xã Chàng Sơn, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I15" t="str">
         <v>hoang.duongminh.1990@hotmail.com</v>
       </c>
-      <c r="G15" t="str">
-        <v>free</v>
-      </c>
-      <c r="H15" t="str">
-        <v>22:00:38 2/6/2026</v>
+      <c r="J15" t="str">
+        <v>free</v>
+      </c>
+      <c r="K15" t="str">
+        <v>02:37:52 3/6/2026</v>
       </c>
     </row>
     <row r="16">
@@ -810,19 +948,28 @@
         <v>11</v>
       </c>
       <c r="D16" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2015-06-04</v>
+      </c>
+      <c r="F16" t="str">
         <v>Lý Văn Tuấn</v>
       </c>
-      <c r="E16">
+      <c r="G16">
         <v>37</v>
       </c>
-      <c r="F16" t="str">
+      <c r="H16" t="str">
+        <v>Phường Viên Sơn, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I16" t="str">
         <v>tuan.lyvan.1989@fpt.edu.vn</v>
       </c>
-      <c r="G16" t="str">
-        <v>free</v>
-      </c>
-      <c r="H16" t="str">
-        <v>18:06:40 12/6/2026</v>
+      <c r="J16" t="str">
+        <v>free</v>
+      </c>
+      <c r="K16" t="str">
+        <v>03:22:12 13/6/2026</v>
       </c>
     </row>
     <row r="17">
@@ -836,19 +983,28 @@
         <v>12</v>
       </c>
       <c r="D17" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2014-01-14</v>
+      </c>
+      <c r="F17" t="str">
         <v>Đinh Văn Hải</v>
       </c>
-      <c r="E17">
+      <c r="G17">
         <v>38</v>
       </c>
-      <c r="F17" t="str">
+      <c r="H17" t="str">
+        <v>Xã Canh Nậu, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I17" t="str">
         <v>hai.dinhvan.1988@gmail.com</v>
       </c>
-      <c r="G17" t="str">
-        <v>free</v>
-      </c>
-      <c r="H17" t="str">
-        <v>01:52:39 18/6/2026</v>
+      <c r="J17" t="str">
+        <v>free</v>
+      </c>
+      <c r="K17" t="str">
+        <v>00:43:11 18/6/2026</v>
       </c>
     </row>
     <row r="18">
@@ -862,19 +1018,28 @@
         <v>5</v>
       </c>
       <c r="D18" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2021-06-27</v>
+      </c>
+      <c r="F18" t="str">
         <v>Lâm Quốc Tuấn</v>
       </c>
-      <c r="E18">
+      <c r="G18">
         <v>39</v>
       </c>
-      <c r="F18" t="str">
+      <c r="H18" t="str">
+        <v>Phường Trung Sơn Trầm, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I18" t="str">
         <v>tuan.lamquoc.1987@yahoo.com</v>
       </c>
-      <c r="G18" t="str">
-        <v>free</v>
-      </c>
-      <c r="H18" t="str">
-        <v>21:11:29 23/5/2026</v>
+      <c r="J18" t="str">
+        <v>free</v>
+      </c>
+      <c r="K18" t="str">
+        <v>21:03:05 23/5/2026</v>
       </c>
     </row>
     <row r="19">
@@ -888,19 +1053,28 @@
         <v>6</v>
       </c>
       <c r="D19" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2020-08-08</v>
+      </c>
+      <c r="F19" t="str">
         <v>Đoàn Văn Hùng</v>
       </c>
-      <c r="E19">
+      <c r="G19">
         <v>40</v>
       </c>
-      <c r="F19" t="str">
+      <c r="H19" t="str">
+        <v>Xã Hữu Bằng, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I19" t="str">
         <v>hung.doanvan.1986@outlook.com</v>
       </c>
-      <c r="G19" t="str">
-        <v>free</v>
-      </c>
-      <c r="H19" t="str">
-        <v>22:21:14 2/6/2026</v>
+      <c r="J19" t="str">
+        <v>free</v>
+      </c>
+      <c r="K19" t="str">
+        <v>23:27:57 2/6/2026</v>
       </c>
     </row>
     <row r="20">
@@ -914,19 +1088,28 @@
         <v>7</v>
       </c>
       <c r="D20" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2019-03-13</v>
+      </c>
+      <c r="F20" t="str">
         <v>Mai Văn Sơn</v>
       </c>
-      <c r="E20">
+      <c r="G20">
         <v>35</v>
       </c>
-      <c r="F20" t="str">
+      <c r="H20" t="str">
+        <v>Xã Đường Lâm, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I20" t="str">
         <v>son.maivan.1991@hotmail.com</v>
       </c>
-      <c r="G20" t="str">
-        <v>free</v>
-      </c>
-      <c r="H20" t="str">
-        <v>02:33:56 13/6/2026</v>
+      <c r="J20" t="str">
+        <v>free</v>
+      </c>
+      <c r="K20" t="str">
+        <v>18:53:09 12/6/2026</v>
       </c>
     </row>
     <row r="21">
@@ -940,19 +1123,28 @@
         <v>8</v>
       </c>
       <c r="D21" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2018-02-18</v>
+      </c>
+      <c r="F21" t="str">
         <v>Trịnh Văn Hải</v>
       </c>
-      <c r="E21">
+      <c r="G21">
         <v>36</v>
       </c>
-      <c r="F21" t="str">
+      <c r="H21" t="str">
+        <v>Xã Thạch Hòa, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I21" t="str">
         <v>hai.trinhvan.1990@fpt.edu.vn</v>
       </c>
-      <c r="G21" t="str">
-        <v>free</v>
-      </c>
-      <c r="H21" t="str">
-        <v>02:23:10 18/6/2026</v>
+      <c r="J21" t="str">
+        <v>free</v>
+      </c>
+      <c r="K21" t="str">
+        <v>21:08:03 17/6/2026</v>
       </c>
     </row>
     <row r="22">
@@ -966,19 +1158,28 @@
         <v>9</v>
       </c>
       <c r="D22" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2017-06-11</v>
+      </c>
+      <c r="F22" t="str">
         <v>Đào Quốc Hưng</v>
       </c>
-      <c r="E22">
+      <c r="G22">
         <v>37</v>
       </c>
-      <c r="F22" t="str">
+      <c r="H22" t="str">
+        <v>Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I22" t="str">
         <v>hung.daoquoc.1989@gmail.com</v>
       </c>
-      <c r="G22" t="str">
-        <v>free</v>
-      </c>
-      <c r="H22" t="str">
-        <v>03:05:10 24/5/2026</v>
+      <c r="J22" t="str">
+        <v>free</v>
+      </c>
+      <c r="K22" t="str">
+        <v>04:04:05 24/5/2026</v>
       </c>
     </row>
     <row r="23">
@@ -992,19 +1193,28 @@
         <v>10</v>
       </c>
       <c r="D23" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2016-04-18</v>
+      </c>
+      <c r="F23" t="str">
         <v>Phùng Văn Hùng</v>
       </c>
-      <c r="E23">
+      <c r="G23">
         <v>38</v>
       </c>
-      <c r="F23" t="str">
+      <c r="H23" t="str">
+        <v>Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I23" t="str">
         <v>hung.phungvan.1988@yahoo.com</v>
       </c>
-      <c r="G23" t="str">
-        <v>free</v>
-      </c>
-      <c r="H23" t="str">
-        <v>01:39:42 3/6/2026</v>
+      <c r="J23" t="str">
+        <v>free</v>
+      </c>
+      <c r="K23" t="str">
+        <v>00:51:33 3/6/2026</v>
       </c>
     </row>
     <row r="24">
@@ -1018,19 +1228,28 @@
         <v>11</v>
       </c>
       <c r="D24" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2015-02-27</v>
+      </c>
+      <c r="F24" t="str">
         <v>Lương Minh Tuấn</v>
       </c>
-      <c r="E24">
+      <c r="G24">
         <v>39</v>
       </c>
-      <c r="F24" t="str">
+      <c r="H24" t="str">
+        <v>TX. Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I24" t="str">
         <v>tuan.luongminh.1987@outlook.com</v>
       </c>
-      <c r="G24" t="str">
-        <v>free</v>
-      </c>
-      <c r="H24" t="str">
-        <v>01:43:55 13/6/2026</v>
+      <c r="J24" t="str">
+        <v>free</v>
+      </c>
+      <c r="K24" t="str">
+        <v>21:47:38 12/6/2026</v>
       </c>
     </row>
     <row r="25">
@@ -1044,19 +1263,28 @@
         <v>12</v>
       </c>
       <c r="D25" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2014-12-08</v>
+      </c>
+      <c r="F25" t="str">
         <v>Đỗ Văn Nam</v>
       </c>
-      <c r="E25">
+      <c r="G25">
         <v>40</v>
       </c>
-      <c r="F25" t="str">
+      <c r="H25" t="str">
+        <v>H. Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I25" t="str">
         <v>nam.dovan.1986@hotmail.com</v>
       </c>
-      <c r="G25" t="str">
-        <v>free</v>
-      </c>
-      <c r="H25" t="str">
-        <v>05:04:25 18/6/2026</v>
+      <c r="J25" t="str">
+        <v>free</v>
+      </c>
+      <c r="K25" t="str">
+        <v>02:10:27 18/6/2026</v>
       </c>
     </row>
     <row r="26">
@@ -1070,19 +1298,28 @@
         <v>5</v>
       </c>
       <c r="D26" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2021-08-08</v>
+      </c>
+      <c r="F26" t="str">
         <v>Nguyễn Văn Dũng</v>
       </c>
-      <c r="E26">
+      <c r="G26">
         <v>35</v>
       </c>
-      <c r="F26" t="str">
+      <c r="H26" t="str">
+        <v>Phường Ngô Quyền, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I26" t="str">
         <v>dung.nguyenvan.1991@fpt.edu.vn</v>
       </c>
-      <c r="G26" t="str">
-        <v>free</v>
-      </c>
-      <c r="H26" t="str">
-        <v>19:58:39 23/5/2026</v>
+      <c r="J26" t="str">
+        <v>free</v>
+      </c>
+      <c r="K26" t="str">
+        <v>02:23:45 24/5/2026</v>
       </c>
     </row>
     <row r="27">
@@ -1096,19 +1333,28 @@
         <v>6</v>
       </c>
       <c r="D27" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2020-08-07</v>
+      </c>
+      <c r="F27" t="str">
         <v>Trần Văn Hùng</v>
       </c>
-      <c r="E27">
+      <c r="G27">
         <v>36</v>
       </c>
-      <c r="F27" t="str">
+      <c r="H27" t="str">
+        <v>Xã Bình Yên, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I27" t="str">
         <v>hung.tranvan.1990@gmail.com</v>
       </c>
-      <c r="G27" t="str">
-        <v>free</v>
-      </c>
-      <c r="H27" t="str">
-        <v>04:35:32 3/6/2026</v>
+      <c r="J27" t="str">
+        <v>free</v>
+      </c>
+      <c r="K27" t="str">
+        <v>00:32:38 3/6/2026</v>
       </c>
     </row>
     <row r="28">
@@ -1122,19 +1368,28 @@
         <v>7</v>
       </c>
       <c r="D28" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2019-05-12</v>
+      </c>
+      <c r="F28" t="str">
         <v>Lê Quốc Huy</v>
       </c>
-      <c r="E28">
+      <c r="G28">
         <v>37</v>
       </c>
-      <c r="F28" t="str">
+      <c r="H28" t="str">
+        <v>Phường Quang Trung, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I28" t="str">
         <v>huy.lequoc.1989@yahoo.com</v>
       </c>
-      <c r="G28" t="str">
-        <v>free</v>
-      </c>
-      <c r="H28" t="str">
-        <v>03:05:31 13/6/2026</v>
+      <c r="J28" t="str">
+        <v>free</v>
+      </c>
+      <c r="K28" t="str">
+        <v>21:53:23 12/6/2026</v>
       </c>
     </row>
     <row r="29">
@@ -1148,19 +1403,28 @@
         <v>8</v>
       </c>
       <c r="D29" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2018-01-17</v>
+      </c>
+      <c r="F29" t="str">
         <v>Phạm Văn Hải</v>
       </c>
-      <c r="E29">
+      <c r="G29">
         <v>38</v>
       </c>
-      <c r="F29" t="str">
+      <c r="H29" t="str">
+        <v>Xã Liên Quan, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I29" t="str">
         <v>hai.phamvan.1988@outlook.com</v>
       </c>
-      <c r="G29" t="str">
-        <v>free</v>
-      </c>
-      <c r="H29" t="str">
-        <v>02:26:16 18/6/2026</v>
+      <c r="J29" t="str">
+        <v>free</v>
+      </c>
+      <c r="K29" t="str">
+        <v>19:53:56 17/6/2026</v>
       </c>
     </row>
     <row r="30">
@@ -1174,19 +1438,28 @@
         <v>9</v>
       </c>
       <c r="D30" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2017-01-18</v>
+      </c>
+      <c r="F30" t="str">
         <v>Vũ Anh Tuấn</v>
       </c>
-      <c r="E30">
+      <c r="G30">
         <v>39</v>
       </c>
-      <c r="F30" t="str">
+      <c r="H30" t="str">
+        <v>Phường Lê Lợi, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I30" t="str">
         <v>tuan.vuanh.1987@hotmail.com</v>
       </c>
-      <c r="G30" t="str">
-        <v>free</v>
-      </c>
-      <c r="H30" t="str">
-        <v>23:43:21 23/5/2026</v>
+      <c r="J30" t="str">
+        <v>free</v>
+      </c>
+      <c r="K30" t="str">
+        <v>23:51:16 23/5/2026</v>
       </c>
     </row>
     <row r="31">
@@ -1200,19 +1473,28 @@
         <v>10</v>
       </c>
       <c r="D31" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2016-08-28</v>
+      </c>
+      <c r="F31" t="str">
         <v>Đặng Quốc Anh</v>
       </c>
-      <c r="E31">
+      <c r="G31">
         <v>40</v>
       </c>
-      <c r="F31" t="str">
+      <c r="H31" t="str">
+        <v>Xã Kim Quan, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I31" t="str">
         <v>anh.dangquoc.1986@fpt.edu.vn</v>
       </c>
-      <c r="G31" t="str">
-        <v>free</v>
-      </c>
-      <c r="H31" t="str">
-        <v>18:44:48 2/6/2026</v>
+      <c r="J31" t="str">
+        <v>free</v>
+      </c>
+      <c r="K31" t="str">
+        <v>01:51:49 3/6/2026</v>
       </c>
     </row>
     <row r="32">
@@ -1226,19 +1508,28 @@
         <v>11</v>
       </c>
       <c r="D32" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2015-05-23</v>
+      </c>
+      <c r="F32" t="str">
         <v>Bùi Văn Hùng</v>
       </c>
-      <c r="E32">
+      <c r="G32">
         <v>35</v>
       </c>
-      <c r="F32" t="str">
+      <c r="H32" t="str">
+        <v>Phường Sơn Lộc, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I32" t="str">
         <v>hung.buivan.1991@gmail.com</v>
       </c>
-      <c r="G32" t="str">
-        <v>free</v>
-      </c>
-      <c r="H32" t="str">
-        <v>04:24:19 13/6/2026</v>
+      <c r="J32" t="str">
+        <v>free</v>
+      </c>
+      <c r="K32" t="str">
+        <v>20:54:00 12/6/2026</v>
       </c>
     </row>
     <row r="33">
@@ -1252,19 +1543,28 @@
         <v>12</v>
       </c>
       <c r="D33" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2014-07-08</v>
+      </c>
+      <c r="F33" t="str">
         <v>Hồ Minh Tuấn</v>
       </c>
-      <c r="E33">
+      <c r="G33">
         <v>36</v>
       </c>
-      <c r="F33" t="str">
+      <c r="H33" t="str">
+        <v>Xã Phùng Xá, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I33" t="str">
         <v>tuan.hominh.1990@yahoo.com</v>
       </c>
-      <c r="G33" t="str">
-        <v>free</v>
-      </c>
-      <c r="H33" t="str">
-        <v>00:43:08 18/6/2026</v>
+      <c r="J33" t="str">
+        <v>free</v>
+      </c>
+      <c r="K33" t="str">
+        <v>03:35:18 18/6/2026</v>
       </c>
     </row>
     <row r="34">
@@ -1278,19 +1578,28 @@
         <v>5</v>
       </c>
       <c r="D34" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2021-05-12</v>
+      </c>
+      <c r="F34" t="str">
         <v>Nguyễn Văn Sơn</v>
       </c>
-      <c r="E34">
+      <c r="G34">
         <v>37</v>
       </c>
-      <c r="F34" t="str">
+      <c r="H34" t="str">
+        <v>Phường Trung Hưng, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I34" t="str">
         <v>son.nguyenvan.1989@outlook.com</v>
       </c>
-      <c r="G34" t="str">
-        <v>free</v>
-      </c>
-      <c r="H34" t="str">
-        <v>22:34:44 23/5/2026</v>
+      <c r="J34" t="str">
+        <v>free</v>
+      </c>
+      <c r="K34" t="str">
+        <v>00:02:23 24/5/2026</v>
       </c>
     </row>
     <row r="35">
@@ -1304,19 +1613,28 @@
         <v>6</v>
       </c>
       <c r="D35" t="str">
+        <v>Nữ</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2020-01-27</v>
+      </c>
+      <c r="F35" t="str">
         <v>Phan Văn Hải</v>
       </c>
-      <c r="E35">
+      <c r="G35">
         <v>38</v>
       </c>
-      <c r="F35" t="str">
+      <c r="H35" t="str">
+        <v>Xã Chàng Sơn, Thạch Thất, Hà Nội</v>
+      </c>
+      <c r="I35" t="str">
         <v>hai.phanvan.1988@hotmail.com</v>
       </c>
-      <c r="G35" t="str">
-        <v>free</v>
-      </c>
-      <c r="H35" t="str">
-        <v>01:07:43 3/6/2026</v>
+      <c r="J35" t="str">
+        <v>free</v>
+      </c>
+      <c r="K35" t="str">
+        <v>19:19:43 2/6/2026</v>
       </c>
     </row>
     <row r="36">
@@ -1330,24 +1648,33 @@
         <v>7</v>
       </c>
       <c r="D36" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2019-11-06</v>
+      </c>
+      <c r="F36" t="str">
         <v>Đỗ Văn Hùng</v>
       </c>
-      <c r="E36">
+      <c r="G36">
         <v>39</v>
       </c>
-      <c r="F36" t="str">
+      <c r="H36" t="str">
+        <v>Phường Viên Sơn, Sơn Tây, Hà Nội</v>
+      </c>
+      <c r="I36" t="str">
         <v>hung.dovan.1987@fpt.edu.vn</v>
       </c>
-      <c r="G36" t="str">
-        <v>free</v>
-      </c>
-      <c r="H36" t="str">
-        <v>01:34:11 13/6/2026</v>
+      <c r="J36" t="str">
+        <v>free</v>
+      </c>
+      <c r="K36" t="str">
+        <v>04:11:32 13/6/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>